<commit_message>
feat(procedures): implementar tags 1 a 5 no radar chart FOR.141 e modulo web para associar perguntas a procedimentos criticos
</commit_message>
<xml_diff>
--- a/FOR.141.r02_Auto_Avaliação.xlsx
+++ b/FOR.141.r02_Auto_Avaliação.xlsx
@@ -614,7 +614,7 @@
               <a:ea typeface="Verdana" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
               <a:cs typeface="Verdana" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>Digite Aqui as perguntas para Avaliação do Treinamento</a:t>
+            <a:t>{{PER_1}}</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -2624,7 +2624,7 @@
               <a:ea typeface="Verdana" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
               <a:cs typeface="Verdana" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>Digite Aqui as perguntas para Avaliação do Treinamento</a:t>
+            <a:t>{{PER_2}}</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -2687,7 +2687,7 @@
               <a:ea typeface="Verdana" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
               <a:cs typeface="Verdana" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>Digite Aqui as perguntas para Avaliação do Treinamento</a:t>
+            <a:t>{{PER_3}}</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -2750,7 +2750,7 @@
               <a:ea typeface="Verdana" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
               <a:cs typeface="Verdana" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>Digite Aqui as perguntas para Avaliação do Treinamento</a:t>
+            <a:t>{{PER_4}}</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -2813,7 +2813,7 @@
               <a:ea typeface="Verdana" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
               <a:cs typeface="Verdana" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t>Digite Aqui as perguntas para Avaliação do Treinamento</a:t>
+            <a:t>{{PER_5}}</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>

</xml_diff>